<commit_message>
revision for site protection and central europ overview.
</commit_message>
<xml_diff>
--- a/map.xlsx
+++ b/map.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mendelu-my.sharepoint.com/personal/xstoces_mendelu_cz1/Documents/SSD_21.12.2024/Kula_Beskydy/2007_2008/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dominik\Beskydy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C5EF9435-C8B4-4C1E-8472-B604EAA98739}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B706D0F8-3A60-486E-9F34-BB67E4FB27D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1275" yWindow="1365" windowWidth="24000" windowHeight="17745" xr2:uid="{C4A6FA0A-7A2B-48B0-977B-2F9F414F2816}"/>
+    <workbookView xWindow="27915" yWindow="1860" windowWidth="23955" windowHeight="15345" xr2:uid="{C4A6FA0A-7A2B-48B0-977B-2F9F414F2816}"/>
   </bookViews>
   <sheets>
     <sheet name="List1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="46">
   <si>
     <t>GPS</t>
   </si>
@@ -165,13 +165,22 @@
   </si>
   <si>
     <t>Beech</t>
+  </si>
+  <si>
+    <t>Site.protection</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Yes</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -200,19 +209,21 @@
       <name val="Lucida Console"/>
       <family val="3"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <charset val="238"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -224,29 +235,36 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normální" xfId="0" builtinId="0"/>
+    <cellStyle name="Normální 2" xfId="1" xr:uid="{A87A62C2-DBC9-44B5-B509-DBDF8A10D01E}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -578,7 +596,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{990468CF-336D-4E81-8C5B-43C805DCE2D9}">
-  <dimension ref="A1:G40"/>
+  <dimension ref="A1:H42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
@@ -596,6 +614,9 @@
       <c r="C1" t="s">
         <v>40</v>
       </c>
+      <c r="D1" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
@@ -607,6 +628,9 @@
       <c r="C2" t="s">
         <v>41</v>
       </c>
+      <c r="D2" s="5" t="s">
+        <v>44</v>
+      </c>
       <c r="G2" s="4"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -619,6 +643,9 @@
       <c r="C3" t="s">
         <v>42</v>
       </c>
+      <c r="D3" s="5" t="s">
+        <v>44</v>
+      </c>
       <c r="G3" s="4"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -631,6 +658,9 @@
       <c r="C4" t="s">
         <v>42</v>
       </c>
+      <c r="D4" s="5" t="s">
+        <v>44</v>
+      </c>
       <c r="G4" s="4"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -643,6 +673,9 @@
       <c r="C5" t="s">
         <v>41</v>
       </c>
+      <c r="D5" s="5" t="s">
+        <v>44</v>
+      </c>
       <c r="G5" s="4"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -655,6 +688,9 @@
       <c r="C6" t="s">
         <v>42</v>
       </c>
+      <c r="D6" s="5" t="s">
+        <v>44</v>
+      </c>
       <c r="G6" s="4"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -667,6 +703,9 @@
       <c r="C7" t="s">
         <v>42</v>
       </c>
+      <c r="D7" s="5" t="s">
+        <v>45</v>
+      </c>
       <c r="G7" s="4"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -679,6 +718,9 @@
       <c r="C8" t="s">
         <v>42</v>
       </c>
+      <c r="D8" s="5" t="s">
+        <v>45</v>
+      </c>
       <c r="G8" s="4"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -691,6 +733,9 @@
       <c r="C9" t="s">
         <v>41</v>
       </c>
+      <c r="D9" s="5" t="s">
+        <v>44</v>
+      </c>
       <c r="G9" s="4"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -703,6 +748,9 @@
       <c r="C10" t="s">
         <v>41</v>
       </c>
+      <c r="D10" s="5" t="s">
+        <v>44</v>
+      </c>
       <c r="G10" s="4"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -715,6 +763,9 @@
       <c r="C11" t="s">
         <v>41</v>
       </c>
+      <c r="D11" s="5" t="s">
+        <v>44</v>
+      </c>
       <c r="G11" s="4"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -727,6 +778,9 @@
       <c r="C12" t="s">
         <v>41</v>
       </c>
+      <c r="D12" s="5" t="s">
+        <v>44</v>
+      </c>
       <c r="G12" s="4"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -739,6 +793,9 @@
       <c r="C13" t="s">
         <v>42</v>
       </c>
+      <c r="D13" s="5" t="s">
+        <v>45</v>
+      </c>
       <c r="G13" s="4"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -751,6 +808,9 @@
       <c r="C14" t="s">
         <v>41</v>
       </c>
+      <c r="D14" s="5" t="s">
+        <v>44</v>
+      </c>
       <c r="G14" s="4"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -763,6 +823,9 @@
       <c r="C15" t="s">
         <v>41</v>
       </c>
+      <c r="D15" s="5" t="s">
+        <v>44</v>
+      </c>
       <c r="G15" s="4"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
@@ -775,6 +838,9 @@
       <c r="C16" t="s">
         <v>41</v>
       </c>
+      <c r="D16" s="5" t="s">
+        <v>44</v>
+      </c>
       <c r="G16" s="4"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -787,6 +853,9 @@
       <c r="C17" t="s">
         <v>41</v>
       </c>
+      <c r="D17" s="5" t="s">
+        <v>44</v>
+      </c>
       <c r="G17" s="4"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
@@ -799,6 +868,9 @@
       <c r="C18" t="s">
         <v>41</v>
       </c>
+      <c r="D18" s="5" t="s">
+        <v>44</v>
+      </c>
       <c r="G18" s="4"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -811,6 +883,9 @@
       <c r="C19" t="s">
         <v>41</v>
       </c>
+      <c r="D19" s="5" t="s">
+        <v>44</v>
+      </c>
       <c r="G19" s="4"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
@@ -823,6 +898,9 @@
       <c r="C20" t="s">
         <v>41</v>
       </c>
+      <c r="D20" s="5" t="s">
+        <v>45</v>
+      </c>
       <c r="G20" s="4"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
@@ -835,6 +913,9 @@
       <c r="C21" t="s">
         <v>41</v>
       </c>
+      <c r="D21" s="5" t="s">
+        <v>45</v>
+      </c>
       <c r="G21" s="4"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
@@ -847,6 +928,9 @@
       <c r="C22" t="s">
         <v>42</v>
       </c>
+      <c r="D22" s="5" t="s">
+        <v>44</v>
+      </c>
       <c r="G22" s="4"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
@@ -859,6 +943,9 @@
       <c r="C23" t="s">
         <v>41</v>
       </c>
+      <c r="D23" s="5" t="s">
+        <v>44</v>
+      </c>
       <c r="G23" s="4"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
@@ -871,6 +958,9 @@
       <c r="C24" t="s">
         <v>41</v>
       </c>
+      <c r="D24" s="5" t="s">
+        <v>44</v>
+      </c>
       <c r="G24" s="4"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
@@ -883,6 +973,9 @@
       <c r="C25" t="s">
         <v>41</v>
       </c>
+      <c r="D25" s="5" t="s">
+        <v>44</v>
+      </c>
       <c r="G25" s="4"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
@@ -895,6 +988,9 @@
       <c r="C26" t="s">
         <v>42</v>
       </c>
+      <c r="D26" s="5" t="s">
+        <v>44</v>
+      </c>
       <c r="G26" s="4"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
@@ -907,6 +1003,9 @@
       <c r="C27" t="s">
         <v>41</v>
       </c>
+      <c r="D27" s="5" t="s">
+        <v>44</v>
+      </c>
       <c r="G27" s="4"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
@@ -919,6 +1018,9 @@
       <c r="C28" t="s">
         <v>42</v>
       </c>
+      <c r="D28" s="5" t="s">
+        <v>44</v>
+      </c>
       <c r="G28" s="4"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
@@ -931,6 +1033,9 @@
       <c r="C29" t="s">
         <v>42</v>
       </c>
+      <c r="D29" s="5" t="s">
+        <v>44</v>
+      </c>
       <c r="G29" s="4"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
@@ -943,6 +1048,9 @@
       <c r="C30" t="s">
         <v>41</v>
       </c>
+      <c r="D30" s="5" t="s">
+        <v>44</v>
+      </c>
       <c r="G30" s="4"/>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
@@ -955,6 +1063,9 @@
       <c r="C31" t="s">
         <v>41</v>
       </c>
+      <c r="D31" s="5" t="s">
+        <v>44</v>
+      </c>
       <c r="G31" s="4"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
@@ -967,9 +1078,12 @@
       <c r="C32" t="s">
         <v>41</v>
       </c>
+      <c r="D32" s="5" t="s">
+        <v>45</v>
+      </c>
       <c r="G32" s="4"/>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
         <v>32</v>
       </c>
@@ -979,9 +1093,12 @@
       <c r="C33" t="s">
         <v>41</v>
       </c>
+      <c r="D33" s="5" t="s">
+        <v>45</v>
+      </c>
       <c r="G33" s="4"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
         <v>33</v>
       </c>
@@ -991,9 +1108,12 @@
       <c r="C34" t="s">
         <v>41</v>
       </c>
+      <c r="D34" s="5" t="s">
+        <v>44</v>
+      </c>
       <c r="G34" s="4"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
         <v>34</v>
       </c>
@@ -1003,9 +1123,12 @@
       <c r="C35" t="s">
         <v>41</v>
       </c>
+      <c r="D35" s="5" t="s">
+        <v>45</v>
+      </c>
       <c r="G35" s="4"/>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
         <v>35</v>
       </c>
@@ -1015,9 +1138,12 @@
       <c r="C36" t="s">
         <v>42</v>
       </c>
+      <c r="D36" s="5" t="s">
+        <v>44</v>
+      </c>
       <c r="G36" s="4"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
         <v>36</v>
       </c>
@@ -1027,9 +1153,12 @@
       <c r="C37" t="s">
         <v>41</v>
       </c>
+      <c r="D37" s="5" t="s">
+        <v>44</v>
+      </c>
       <c r="G37" s="4"/>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
         <v>37</v>
       </c>
@@ -1039,9 +1168,14 @@
       <c r="C38" t="s">
         <v>41</v>
       </c>
-      <c r="G38" s="4"/>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D38" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="F38" s="6"/>
+      <c r="G38" s="7"/>
+      <c r="H38" s="6"/>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
         <v>38</v>
       </c>
@@ -1051,10 +1185,27 @@
       <c r="C39" t="s">
         <v>41</v>
       </c>
-      <c r="G39" s="4"/>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="G40" s="5"/>
+      <c r="D39" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="F39" s="8"/>
+      <c r="G39" s="8"/>
+      <c r="H39" s="8"/>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="F40" s="8"/>
+      <c r="G40" s="8"/>
+      <c r="H40" s="8"/>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="F41" s="8"/>
+      <c r="G41" s="8"/>
+      <c r="H41" s="8"/>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="F42" s="8"/>
+      <c r="G42" s="8"/>
+      <c r="H42" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>

</xml_diff>